<commit_message>
Add PDF-based lease skill; convert Ironhide lease to PDF; revert DB rows
</commit_message>
<xml_diff>
--- a/2-build-lease-abstraction/Database.xlsx
+++ b/2-build-lease-abstraction/Database.xlsx
@@ -684,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.6"/>
   <cols>
     <col width="30.53515625" customWidth="1" min="1" max="7"/>
@@ -701,31 +701,6 @@
           <t>tenant_name</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>tenant_entity_type</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>tenant_contact_name</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>tenant_contact_email</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>tenant_contact_phone</t>
-        </is>
-      </c>
-      <c r="G1" s="3" t="inlineStr">
-        <is>
-          <t>notes</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -734,11 +709,6 @@
         </is>
       </c>
       <c r="B2" s="5" t="n"/>
-      <c r="C2" s="5" t="n"/>
-      <c r="D2" s="5" t="n"/>
-      <c r="E2" s="5" t="n"/>
-      <c r="F2" s="5" t="n"/>
-      <c r="G2" s="6" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -751,31 +721,6 @@
           <t>string</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="G3" s="9" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
     </row>
     <row r="4" ht="50.05" customHeight="1">
       <c r="A4" s="10" t="inlineStr">
@@ -786,66 +731,6 @@
       <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Legal name of occupying entity</t>
-        </is>
-      </c>
-      <c r="C4" s="11" t="inlineStr">
-        <is>
-          <t>LLC, Corp, Individual, etc.</t>
-        </is>
-      </c>
-      <c r="D4" s="11" t="inlineStr">
-        <is>
-          <t>Primary contact person</t>
-        </is>
-      </c>
-      <c r="E4" s="11" t="inlineStr">
-        <is>
-          <t>Primary contact email</t>
-        </is>
-      </c>
-      <c r="F4" s="11" t="inlineStr">
-        <is>
-          <t>Primary contact phone</t>
-        </is>
-      </c>
-      <c r="G4" s="12" t="inlineStr">
-        <is>
-          <t>Free-text notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Ironhide Cold Logistics, LLC</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>LLC</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Hjalmar P. Lindqvist</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>hlindqvist@ironhidecold.example</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>(801) 555-0418</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Delaware LLC, authorized to do business in Utah. Director of Operations is primary contact. 24/7 ammonia/spill/emergency line (801) 555-0911.</t>
         </is>
       </c>
     </row>
@@ -861,7 +746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.6"/>
   <cols>
     <col width="30.53515625" customWidth="1" min="1" max="7"/>
@@ -878,31 +763,6 @@
           <t>landlord_name</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>landlord_entity_type</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>landlord_contact_name</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>landlord_contact_email</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>landlord_contact_phone</t>
-        </is>
-      </c>
-      <c r="G1" s="3" t="inlineStr">
-        <is>
-          <t>notes</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -911,11 +771,6 @@
         </is>
       </c>
       <c r="B2" s="5" t="n"/>
-      <c r="C2" s="5" t="n"/>
-      <c r="D2" s="5" t="n"/>
-      <c r="E2" s="5" t="n"/>
-      <c r="F2" s="5" t="n"/>
-      <c r="G2" s="6" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -928,31 +783,6 @@
           <t>string</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="G3" s="9" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
     </row>
     <row r="4" ht="50.05" customHeight="1">
       <c r="A4" s="10" t="inlineStr">
@@ -963,62 +793,6 @@
       <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Legal name of owning/leasing entity</t>
-        </is>
-      </c>
-      <c r="C4" s="11" t="inlineStr">
-        <is>
-          <t>LLC, REIT, Trust, etc.</t>
-        </is>
-      </c>
-      <c r="D4" s="11" t="inlineStr">
-        <is>
-          <t>Primary contact person</t>
-        </is>
-      </c>
-      <c r="E4" s="11" t="inlineStr">
-        <is>
-          <t>Primary contact email</t>
-        </is>
-      </c>
-      <c r="F4" s="11" t="inlineStr">
-        <is>
-          <t>Primary contact phone</t>
-        </is>
-      </c>
-      <c r="G4" s="12" t="inlineStr">
-        <is>
-          <t>Free-text notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Beehive Realty Trust, LLC</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>LLC</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Lease Administration</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>leases@beehiverealtytrust.example</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Utah LLC; landlord broker handled in-house (Beehive Realty Trust, LLC). Notice address: 175 East 400 South, Suite 900, Salt Lake City, UT 84111.</t>
         </is>
       </c>
     </row>
@@ -1034,7 +808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.6"/>
   <cols>
     <col width="30.53515625" customWidth="1" min="1" max="6"/>
@@ -1066,11 +840,6 @@
           <t>size_unit</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
-        <is>
-          <t>notes</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -1090,7 +859,6 @@
           <t>CHECK constraint</t>
         </is>
       </c>
-      <c r="F2" s="6" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -1118,11 +886,6 @@
           <t>enum: RSF, ACRE</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
     </row>
     <row r="4" ht="50.05" customHeight="1">
       <c r="A4" s="10" t="inlineStr">
@@ -1148,39 +911,6 @@
       <c r="E4" s="11" t="inlineStr">
         <is>
           <t>Unit for size (RSF rentable sq ft, ACRE acres)</t>
-        </is>
-      </c>
-      <c r="F4" s="12" t="inlineStr">
-        <is>
-          <t>Free-text notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>4280 West Indiana Avenue, West Valley City, UT 84120</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>IND</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>88500</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>RSF</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Single-tenant cold-storage warehouse on approx. 6.1 acres; whole-building lease. 36-ft clear height; NH3 refrigeration plant, under-slab heating, 32 dock doors, 1 drive-in door, 2 rail-service doors (Union Pacific spur), 24 reefer stalls with 480V plug-ins.</t>
         </is>
       </c>
     </row>
@@ -1196,7 +926,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.6"/>
   <cols>
     <col width="31.3828125" customWidth="1" min="1" max="15"/>
@@ -1250,32 +980,22 @@
       </c>
       <c r="J1" s="14" t="inlineStr">
         <is>
-          <t>base_rent_frequency</t>
+          <t>escalation_pct</t>
         </is>
       </c>
       <c r="K1" s="14" t="inlineStr">
         <is>
-          <t>escalation_pct</t>
+          <t>security_deposit_amount</t>
         </is>
       </c>
       <c r="L1" s="14" t="inlineStr">
         <is>
-          <t>security_deposit_amount</t>
+          <t>security_deposit_type</t>
         </is>
       </c>
       <c r="M1" s="14" t="inlineStr">
         <is>
-          <t>security_deposit_type</t>
-        </is>
-      </c>
-      <c r="N1" s="14" t="inlineStr">
-        <is>
           <t>permitted_use</t>
-        </is>
-      </c>
-      <c r="O1" s="15" t="inlineStr">
-        <is>
-          <t>notes</t>
         </is>
       </c>
     </row>
@@ -1311,14 +1031,12 @@
       <c r="I2" s="5" t="n"/>
       <c r="J2" s="5" t="n"/>
       <c r="K2" s="5" t="n"/>
-      <c r="L2" s="5" t="n"/>
-      <c r="M2" s="5" t="inlineStr">
+      <c r="L2" s="5" t="inlineStr">
         <is>
           <t>CHECK constraint</t>
         </is>
       </c>
-      <c r="N2" s="5" t="n"/>
-      <c r="O2" s="6" t="n"/>
+      <c r="M2" s="5" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -1368,30 +1086,20 @@
       </c>
       <c r="J3" s="8" t="inlineStr">
         <is>
-          <t>enum (ANNUAL/MONTHLY)</t>
+          <t>decimal (percent)</t>
         </is>
       </c>
       <c r="K3" s="8" t="inlineStr">
         <is>
-          <t>decimal (percent)</t>
+          <t>decimal (currency)</t>
         </is>
       </c>
       <c r="L3" s="8" t="inlineStr">
         <is>
-          <t>decimal (currency)</t>
+          <t>enum: Cash, CL, NONE</t>
         </is>
       </c>
       <c r="M3" s="8" t="inlineStr">
-        <is>
-          <t>enum: Cash, CL, NONE</t>
-        </is>
-      </c>
-      <c r="N3" s="8" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="O3" s="9" t="inlineStr">
         <is>
           <t>string</t>
         </is>
@@ -1445,93 +1153,22 @@
       </c>
       <c r="J4" s="11" t="inlineStr">
         <is>
-          <t>Whether base_rent is annual or monthly</t>
+          <t>Annual step-up percentage</t>
         </is>
       </c>
       <c r="K4" s="11" t="inlineStr">
         <is>
-          <t>Annual step-up percentage</t>
+          <t>Deposit value</t>
         </is>
       </c>
       <c r="L4" s="11" t="inlineStr">
         <is>
-          <t>Deposit value</t>
+          <t>Form of deposit (Cash cash deposit, CL letter of credit, NONE none)</t>
         </is>
       </c>
       <c r="M4" s="11" t="inlineStr">
         <is>
-          <t>Form of deposit (Cash cash deposit, CL letter of credit, NONE none)</t>
-        </is>
-      </c>
-      <c r="N4" s="11" t="inlineStr">
-        <is>
           <t>Allowed use of the space</t>
-        </is>
-      </c>
-      <c r="O4" s="12" t="inlineStr">
-        <is>
-          <t>Free-text notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" t="n">
-        <v>1</v>
-      </c>
-      <c r="C5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>2036-11-30</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
-        <v>120</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>NNN</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>1283250</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>ANNUAL</t>
-        </is>
-      </c>
-      <c r="K5" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="L5" t="n">
-        <v>641625</v>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Refrigerated/frozen warehousing, storage, cross-docking, blast-freezing, ambient warehousing, value-added repack, customer-pick logistics, transportation management, and ancillary office, in support of 3PL operations.</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>Base Rent abated Dec 1, 2026 - Mar 31, 2027 (rent commences Apr 1, 2027). ~2.5% annual escalation ($14.50 -&gt; $18.10 per RSF). Recorded base_rent is the first full (non-abated) annual rate. Security is a $641,625 irrevocable standby LC (no cash deposit), with burn-down per Section 2.7 ($480k at Y+1, $320k at Y+3, $160k at Y+5). Estimated NNN $4.20/RSF (2027); $15/RSF TI allowance ($1,327,500).</t>
         </is>
       </c>
     </row>
@@ -1547,7 +1184,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.6"/>
   <cols>
     <col width="31.3828125" customWidth="1" min="1" max="9"/>
@@ -1581,22 +1218,12 @@
       </c>
       <c r="F1" s="14" t="inlineStr">
         <is>
-          <t>renewal_rent_value</t>
+          <t>notice_min_months</t>
         </is>
       </c>
       <c r="G1" s="14" t="inlineStr">
         <is>
-          <t>notice_min_months</t>
-        </is>
-      </c>
-      <c r="H1" s="14" t="inlineStr">
-        <is>
           <t>notice_max_months</t>
-        </is>
-      </c>
-      <c r="I1" s="15" t="inlineStr">
-        <is>
-          <t>notes</t>
         </is>
       </c>
     </row>
@@ -1620,8 +1247,6 @@
       </c>
       <c r="F2" s="5" t="n"/>
       <c r="G2" s="5" t="n"/>
-      <c r="H2" s="5" t="n"/>
-      <c r="I2" s="6" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -1651,22 +1276,12 @@
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t>decimal (currency or percent)</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr">
         <is>
           <t>integer</t>
-        </is>
-      </c>
-      <c r="H3" s="8" t="inlineStr">
-        <is>
-          <t>integer</t>
-        </is>
-      </c>
-      <c r="I3" s="9" t="inlineStr">
-        <is>
-          <t>string</t>
         </is>
       </c>
     </row>
@@ -1698,82 +1313,12 @@
       </c>
       <c r="F4" s="11" t="inlineStr">
         <is>
-          <t>Stated rent if FIX, or CPI cap if CPI</t>
+          <t>Earliest notice before expiry</t>
         </is>
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>Earliest notice before expiry</t>
-        </is>
-      </c>
-      <c r="H4" s="11" t="inlineStr">
-        <is>
           <t>Latest notice before expiry</t>
-        </is>
-      </c>
-      <c r="I4" s="12" t="inlineStr">
-        <is>
-          <t>Free-text notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" t="n">
-        <v>1</v>
-      </c>
-      <c r="C5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" t="n">
-        <v>60</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>FMR</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
-        <v>15</v>
-      </c>
-      <c r="H5" t="n">
-        <v>18</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Notice window: not earlier than 18 months and not later than 15 months before the then-current Expiration Date (Article 27.2). Conditions: no uncured Event of Default; original Tenant (or Permitted Transferee) in occupancy of &gt;=90% of Premises. FMR by appraisal if not agreed in 30 days.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" t="n">
-        <v>1</v>
-      </c>
-      <c r="C6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D6" t="n">
-        <v>60</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>FMR</t>
-        </is>
-      </c>
-      <c r="G6" t="n">
-        <v>15</v>
-      </c>
-      <c r="H6" t="n">
-        <v>18</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Second consecutive 5-year option at Fair Market Rent; same notice window and conditions as option 1. Time of the essence; missing a window terminates that and all later options.</t>
         </is>
       </c>
     </row>

</xml_diff>